<commit_message>
* Correcciones en recibo y en submodulos
</commit_message>
<xml_diff>
--- a/.data/Recibo.xlsx
+++ b/.data/Recibo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox (Personal)\Proyectos\CasaLuna\dev\.data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F83FFC0-BE09-44E1-8726-303DC08DE2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{303F9D44-7D92-4E94-B262-AC897FD248E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="40080" yWindow="-13140" windowWidth="16440" windowHeight="29040" xr2:uid="{7A2361CB-5B98-48A2-B605-CBE71B4933E3}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="46">
   <si>
     <t>{{Cliente}}</t>
   </si>
@@ -92,9 +92,6 @@
     <t>FECHA DE FOTO:</t>
   </si>
   <si>
-    <t>{{anticipo}}</t>
-  </si>
-  <si>
     <t>FOLIO</t>
   </si>
   <si>
@@ -146,9 +143,6 @@
     <t>DESCUENTO</t>
   </si>
   <si>
-    <t>{{descuento}}</t>
-  </si>
-  <si>
     <t>{{suma_subtotal}}</t>
   </si>
   <si>
@@ -165,6 +159,21 @@
   </si>
   <si>
     <t>{{restante}}</t>
+  </si>
+  <si>
+    <t>ANTICIPOS</t>
+  </si>
+  <si>
+    <t>{{anticipos}}</t>
+  </si>
+  <si>
+    <t>XV / NOVIA:</t>
+  </si>
+  <si>
+    <t>{{Festejada}}</t>
+  </si>
+  <si>
+    <t>{{fecha_anticipo}} - {{anticipo}}</t>
   </si>
 </sst>
 </file>
@@ -672,6 +681,93 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -699,143 +795,56 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1428,21 +1437,21 @@
     <row r="6" spans="2:20" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B6" s="4"/>
       <c r="C6" s="5"/>
-      <c r="D6" s="68" t="s">
+      <c r="D6" s="79" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="79"/>
+      <c r="F6" s="79"/>
+      <c r="G6" s="79"/>
+      <c r="H6" s="79"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="93" t="s">
         <v>26</v>
       </c>
-      <c r="E6" s="68"/>
-      <c r="F6" s="68"/>
-      <c r="G6" s="68"/>
-      <c r="H6" s="68"/>
-      <c r="I6" s="8"/>
-      <c r="J6" s="56" t="s">
-        <v>27</v>
-      </c>
-      <c r="K6" s="56"/>
-      <c r="L6" s="56"/>
-      <c r="M6" s="56"/>
-      <c r="N6" s="56"/>
+      <c r="K6" s="93"/>
+      <c r="L6" s="93"/>
+      <c r="M6" s="93"/>
+      <c r="N6" s="93"/>
       <c r="O6" s="5"/>
       <c r="P6" s="5"/>
       <c r="Q6" s="5"/>
@@ -1453,48 +1462,48 @@
     <row r="7" spans="2:20" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="4"/>
       <c r="C7" s="5"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="68"/>
+      <c r="D7" s="79"/>
+      <c r="E7" s="79"/>
+      <c r="F7" s="79"/>
+      <c r="G7" s="79"/>
+      <c r="H7" s="79"/>
       <c r="I7" s="40"/>
-      <c r="J7" s="56"/>
-      <c r="K7" s="56"/>
-      <c r="L7" s="56"/>
-      <c r="M7" s="56"/>
-      <c r="N7" s="56"/>
-      <c r="O7" s="59" t="s">
-        <v>19</v>
-      </c>
-      <c r="P7" s="60"/>
-      <c r="Q7" s="60"/>
-      <c r="R7" s="61"/>
+      <c r="J7" s="93"/>
+      <c r="K7" s="93"/>
+      <c r="L7" s="93"/>
+      <c r="M7" s="93"/>
+      <c r="N7" s="93"/>
+      <c r="O7" s="82" t="s">
+        <v>18</v>
+      </c>
+      <c r="P7" s="83"/>
+      <c r="Q7" s="83"/>
+      <c r="R7" s="84"/>
       <c r="S7" s="17"/>
       <c r="T7" s="6"/>
     </row>
     <row r="8" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="4"/>
       <c r="C8" s="5"/>
-      <c r="D8" s="68"/>
-      <c r="E8" s="68"/>
-      <c r="F8" s="68"/>
-      <c r="G8" s="68"/>
-      <c r="H8" s="68"/>
+      <c r="D8" s="79"/>
+      <c r="E8" s="79"/>
+      <c r="F8" s="79"/>
+      <c r="G8" s="79"/>
+      <c r="H8" s="79"/>
       <c r="I8" s="8"/>
-      <c r="J8" s="56" t="s">
-        <v>30</v>
-      </c>
-      <c r="K8" s="56"/>
-      <c r="L8" s="56"/>
-      <c r="M8" s="56"/>
-      <c r="N8" s="56"/>
-      <c r="O8" s="62" t="s">
-        <v>20</v>
-      </c>
-      <c r="P8" s="63"/>
-      <c r="Q8" s="63"/>
-      <c r="R8" s="64"/>
+      <c r="J8" s="93" t="s">
+        <v>29</v>
+      </c>
+      <c r="K8" s="93"/>
+      <c r="L8" s="93"/>
+      <c r="M8" s="93"/>
+      <c r="N8" s="93"/>
+      <c r="O8" s="85" t="s">
+        <v>19</v>
+      </c>
+      <c r="P8" s="86"/>
+      <c r="Q8" s="86"/>
+      <c r="R8" s="87"/>
       <c r="S8" s="17"/>
       <c r="T8" s="6"/>
     </row>
@@ -1504,18 +1513,18 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="53"/>
-      <c r="H9" s="53"/>
+      <c r="G9" s="49"/>
+      <c r="H9" s="49"/>
       <c r="I9" s="40"/>
-      <c r="J9" s="56"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="56"/>
-      <c r="M9" s="56"/>
-      <c r="N9" s="56"/>
-      <c r="O9" s="65"/>
-      <c r="P9" s="66"/>
-      <c r="Q9" s="66"/>
-      <c r="R9" s="67"/>
+      <c r="J9" s="93"/>
+      <c r="K9" s="93"/>
+      <c r="L9" s="93"/>
+      <c r="M9" s="93"/>
+      <c r="N9" s="93"/>
+      <c r="O9" s="88"/>
+      <c r="P9" s="89"/>
+      <c r="Q9" s="89"/>
+      <c r="R9" s="90"/>
       <c r="S9" s="17"/>
       <c r="T9" s="6"/>
     </row>
@@ -1523,13 +1532,13 @@
       <c r="B10" s="4"/>
       <c r="C10" s="5"/>
       <c r="D10" s="5"/>
-      <c r="E10" s="58" t="s">
+      <c r="E10" s="92" t="s">
+        <v>23</v>
+      </c>
+      <c r="F10" s="92"/>
+      <c r="G10" s="92"/>
+      <c r="H10" s="36" t="s">
         <v>24</v>
-      </c>
-      <c r="F10" s="58"/>
-      <c r="G10" s="58"/>
-      <c r="H10" s="36" t="s">
-        <v>25</v>
       </c>
       <c r="I10" s="8"/>
       <c r="J10" s="36"/>
@@ -1615,23 +1624,23 @@
         <v>12</v>
       </c>
       <c r="F14" s="7"/>
-      <c r="G14" s="54" t="s">
+      <c r="G14" s="94" t="s">
         <v>0</v>
       </c>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="H14" s="94"/>
+      <c r="I14" s="94"/>
       <c r="J14" s="9"/>
       <c r="K14" s="8"/>
-      <c r="L14" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="M14" s="53"/>
-      <c r="N14" s="53"/>
-      <c r="O14" s="55" t="s">
-        <v>40</v>
-      </c>
-      <c r="P14" s="55"/>
-      <c r="Q14" s="55"/>
+      <c r="L14" s="49" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="49"/>
+      <c r="N14" s="49"/>
+      <c r="O14" s="81" t="s">
+        <v>38</v>
+      </c>
+      <c r="P14" s="81"/>
+      <c r="Q14" s="81"/>
       <c r="R14" s="19"/>
       <c r="S14" s="19"/>
       <c r="T14" s="6"/>
@@ -1640,23 +1649,27 @@
       <c r="B15" s="4"/>
       <c r="C15" s="27"/>
       <c r="D15" s="5"/>
-      <c r="E15" s="7"/>
+      <c r="E15" s="7" t="s">
+        <v>43</v>
+      </c>
       <c r="F15" s="7"/>
-      <c r="G15" s="55"/>
-      <c r="H15" s="55"/>
-      <c r="I15" s="55"/>
+      <c r="G15" s="94" t="s">
+        <v>44</v>
+      </c>
+      <c r="H15" s="94"/>
+      <c r="I15" s="94"/>
       <c r="J15" s="9"/>
       <c r="K15" s="8"/>
-      <c r="L15" s="53" t="s">
+      <c r="L15" s="49" t="s">
         <v>15</v>
       </c>
-      <c r="M15" s="53"/>
-      <c r="N15" s="53"/>
-      <c r="O15" s="57" t="s">
-        <v>21</v>
-      </c>
-      <c r="P15" s="57"/>
-      <c r="Q15" s="57"/>
+      <c r="M15" s="49"/>
+      <c r="N15" s="49"/>
+      <c r="O15" s="91" t="s">
+        <v>20</v>
+      </c>
+      <c r="P15" s="91"/>
+      <c r="Q15" s="91"/>
       <c r="R15" s="19"/>
       <c r="S15" s="19"/>
       <c r="T15" s="6"/>
@@ -1669,23 +1682,23 @@
         <v>13</v>
       </c>
       <c r="F16" s="7"/>
-      <c r="G16" s="69" t="s">
-        <v>34</v>
-      </c>
-      <c r="H16" s="69"/>
-      <c r="I16" s="69"/>
+      <c r="G16" s="80" t="s">
+        <v>33</v>
+      </c>
+      <c r="H16" s="80"/>
+      <c r="I16" s="80"/>
       <c r="J16" s="9"/>
       <c r="K16" s="8"/>
-      <c r="L16" s="53" t="s">
+      <c r="L16" s="49" t="s">
         <v>17</v>
       </c>
-      <c r="M16" s="53"/>
-      <c r="N16" s="53"/>
-      <c r="O16" s="57" t="s">
-        <v>22</v>
-      </c>
-      <c r="P16" s="57"/>
-      <c r="Q16" s="57"/>
+      <c r="M16" s="49"/>
+      <c r="N16" s="49"/>
+      <c r="O16" s="91" t="s">
+        <v>21</v>
+      </c>
+      <c r="P16" s="91"/>
+      <c r="Q16" s="91"/>
       <c r="R16" s="19"/>
       <c r="S16" s="19"/>
       <c r="T16" s="6"/>
@@ -1696,21 +1709,21 @@
       <c r="D17" s="5"/>
       <c r="E17" s="7"/>
       <c r="F17" s="7"/>
-      <c r="G17" s="55"/>
-      <c r="H17" s="55"/>
-      <c r="I17" s="55"/>
+      <c r="G17" s="81"/>
+      <c r="H17" s="81"/>
+      <c r="I17" s="81"/>
       <c r="J17" s="9"/>
       <c r="K17" s="8"/>
-      <c r="L17" s="53" t="s">
+      <c r="L17" s="49" t="s">
         <v>16</v>
       </c>
-      <c r="M17" s="53"/>
-      <c r="N17" s="53"/>
-      <c r="O17" s="57" t="s">
-        <v>23</v>
-      </c>
-      <c r="P17" s="57"/>
-      <c r="Q17" s="57"/>
+      <c r="M17" s="49"/>
+      <c r="N17" s="49"/>
+      <c r="O17" s="91" t="s">
+        <v>22</v>
+      </c>
+      <c r="P17" s="91"/>
+      <c r="Q17" s="91"/>
       <c r="R17" s="19"/>
       <c r="S17" s="19"/>
       <c r="T17" s="6"/>
@@ -1723,11 +1736,11 @@
         <v>14</v>
       </c>
       <c r="F18" s="7"/>
-      <c r="G18" s="57" t="s">
-        <v>28</v>
-      </c>
-      <c r="H18" s="57"/>
-      <c r="I18" s="57"/>
+      <c r="G18" s="91" t="s">
+        <v>27</v>
+      </c>
+      <c r="H18" s="91"/>
+      <c r="I18" s="91"/>
       <c r="J18" s="9"/>
       <c r="K18" s="8"/>
       <c r="L18" s="37"/>
@@ -1805,632 +1818,632 @@
     </row>
     <row r="22" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="4"/>
-      <c r="C22" s="71" t="s">
+      <c r="C22" s="50" t="s">
         <v>7</v>
       </c>
-      <c r="D22" s="72"/>
-      <c r="E22" s="72"/>
-      <c r="F22" s="73"/>
-      <c r="G22" s="71" t="s">
+      <c r="D22" s="51"/>
+      <c r="E22" s="51"/>
+      <c r="F22" s="52"/>
+      <c r="G22" s="50" t="s">
         <v>8</v>
       </c>
-      <c r="H22" s="72"/>
-      <c r="I22" s="73"/>
-      <c r="J22" s="71" t="s">
+      <c r="H22" s="51"/>
+      <c r="I22" s="52"/>
+      <c r="J22" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="K22" s="72"/>
-      <c r="L22" s="73"/>
-      <c r="M22" s="71" t="s">
-        <v>35</v>
-      </c>
-      <c r="N22" s="72"/>
-      <c r="O22" s="73"/>
-      <c r="P22" s="71" t="s">
-        <v>32</v>
-      </c>
-      <c r="Q22" s="72"/>
-      <c r="R22" s="72"/>
-      <c r="S22" s="73"/>
+      <c r="K22" s="51"/>
+      <c r="L22" s="52"/>
+      <c r="M22" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="N22" s="51"/>
+      <c r="O22" s="52"/>
+      <c r="P22" s="51" t="s">
+        <v>41</v>
+      </c>
+      <c r="Q22" s="51"/>
+      <c r="R22" s="51"/>
+      <c r="S22" s="52"/>
       <c r="T22" s="6"/>
     </row>
     <row r="23" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B23" s="4"/>
-      <c r="C23" s="74"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
-      <c r="F23" s="76"/>
-      <c r="G23" s="74"/>
-      <c r="H23" s="75"/>
-      <c r="I23" s="76"/>
-      <c r="J23" s="74"/>
-      <c r="K23" s="75"/>
-      <c r="L23" s="76"/>
-      <c r="M23" s="74"/>
-      <c r="N23" s="75"/>
-      <c r="O23" s="76"/>
-      <c r="P23" s="74"/>
-      <c r="Q23" s="75"/>
-      <c r="R23" s="75"/>
-      <c r="S23" s="76"/>
+      <c r="C23" s="57"/>
+      <c r="D23" s="58"/>
+      <c r="E23" s="58"/>
+      <c r="F23" s="59"/>
+      <c r="G23" s="57"/>
+      <c r="H23" s="58"/>
+      <c r="I23" s="59"/>
+      <c r="J23" s="57"/>
+      <c r="K23" s="58"/>
+      <c r="L23" s="59"/>
+      <c r="M23" s="57"/>
+      <c r="N23" s="58"/>
+      <c r="O23" s="59"/>
+      <c r="P23" s="58"/>
+      <c r="Q23" s="58"/>
+      <c r="R23" s="58"/>
+      <c r="S23" s="59"/>
       <c r="T23" s="6"/>
     </row>
     <row r="24" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="4"/>
-      <c r="C24" s="41" t="s">
+      <c r="C24" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D24" s="42"/>
-      <c r="E24" s="42"/>
-      <c r="F24" s="43"/>
-      <c r="G24" s="41" t="s">
+      <c r="D24" s="71"/>
+      <c r="E24" s="71"/>
+      <c r="F24" s="72"/>
+      <c r="G24" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H24" s="42"/>
-      <c r="I24" s="43"/>
-      <c r="J24" s="41" t="s">
+      <c r="H24" s="71"/>
+      <c r="I24" s="72"/>
+      <c r="J24" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K24" s="42"/>
-      <c r="L24" s="43"/>
-      <c r="M24" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N24" s="42"/>
-      <c r="O24" s="43"/>
-      <c r="P24" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q24" s="42"/>
-      <c r="R24" s="42"/>
-      <c r="S24" s="43"/>
+      <c r="K24" s="71"/>
+      <c r="L24" s="72"/>
+      <c r="M24" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N24" s="71"/>
+      <c r="O24" s="72"/>
+      <c r="P24" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q24" s="71"/>
+      <c r="R24" s="71"/>
+      <c r="S24" s="72"/>
       <c r="T24" s="6"/>
     </row>
     <row r="25" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B25" s="4"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="45"/>
-      <c r="E25" s="45"/>
-      <c r="F25" s="46"/>
-      <c r="G25" s="44"/>
-      <c r="H25" s="93"/>
-      <c r="I25" s="46"/>
-      <c r="J25" s="44"/>
-      <c r="K25" s="93"/>
-      <c r="L25" s="46"/>
-      <c r="M25" s="44"/>
-      <c r="N25" s="93"/>
-      <c r="O25" s="46"/>
-      <c r="P25" s="44"/>
-      <c r="Q25" s="45"/>
-      <c r="R25" s="45"/>
-      <c r="S25" s="46"/>
+      <c r="C25" s="73"/>
+      <c r="D25" s="74"/>
+      <c r="E25" s="74"/>
+      <c r="F25" s="75"/>
+      <c r="G25" s="73"/>
+      <c r="H25" s="74"/>
+      <c r="I25" s="75"/>
+      <c r="J25" s="73"/>
+      <c r="K25" s="74"/>
+      <c r="L25" s="75"/>
+      <c r="M25" s="73"/>
+      <c r="N25" s="74"/>
+      <c r="O25" s="75"/>
+      <c r="P25" s="95"/>
+      <c r="Q25" s="95"/>
+      <c r="R25" s="95"/>
+      <c r="S25" s="75"/>
       <c r="T25" s="6"/>
     </row>
     <row r="26" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B26" s="4"/>
-      <c r="C26" s="47"/>
-      <c r="D26" s="48"/>
-      <c r="E26" s="48"/>
-      <c r="F26" s="49"/>
-      <c r="G26" s="47"/>
-      <c r="H26" s="48"/>
-      <c r="I26" s="49"/>
-      <c r="J26" s="47"/>
-      <c r="K26" s="48"/>
-      <c r="L26" s="49"/>
-      <c r="M26" s="47"/>
-      <c r="N26" s="48"/>
-      <c r="O26" s="49"/>
-      <c r="P26" s="47"/>
-      <c r="Q26" s="48"/>
-      <c r="R26" s="48"/>
-      <c r="S26" s="49"/>
+      <c r="C26" s="76"/>
+      <c r="D26" s="77"/>
+      <c r="E26" s="77"/>
+      <c r="F26" s="78"/>
+      <c r="G26" s="76"/>
+      <c r="H26" s="77"/>
+      <c r="I26" s="78"/>
+      <c r="J26" s="76"/>
+      <c r="K26" s="77"/>
+      <c r="L26" s="78"/>
+      <c r="M26" s="76"/>
+      <c r="N26" s="77"/>
+      <c r="O26" s="78"/>
+      <c r="P26" s="77"/>
+      <c r="Q26" s="77"/>
+      <c r="R26" s="77"/>
+      <c r="S26" s="78"/>
       <c r="T26" s="6"/>
     </row>
     <row r="27" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B27" s="4"/>
-      <c r="C27" s="41" t="s">
+      <c r="C27" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D27" s="42"/>
-      <c r="E27" s="42"/>
-      <c r="F27" s="43"/>
-      <c r="G27" s="41" t="s">
+      <c r="D27" s="71"/>
+      <c r="E27" s="71"/>
+      <c r="F27" s="72"/>
+      <c r="G27" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H27" s="42"/>
-      <c r="I27" s="43"/>
-      <c r="J27" s="41" t="s">
+      <c r="H27" s="71"/>
+      <c r="I27" s="72"/>
+      <c r="J27" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K27" s="42"/>
-      <c r="L27" s="43"/>
-      <c r="M27" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N27" s="42"/>
-      <c r="O27" s="43"/>
-      <c r="P27" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q27" s="42"/>
-      <c r="R27" s="42"/>
-      <c r="S27" s="43"/>
+      <c r="K27" s="71"/>
+      <c r="L27" s="72"/>
+      <c r="M27" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N27" s="71"/>
+      <c r="O27" s="72"/>
+      <c r="P27" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q27" s="71"/>
+      <c r="R27" s="71"/>
+      <c r="S27" s="72"/>
       <c r="T27" s="6"/>
     </row>
     <row r="28" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B28" s="4"/>
-      <c r="C28" s="44"/>
-      <c r="D28" s="45"/>
-      <c r="E28" s="45"/>
-      <c r="F28" s="46"/>
-      <c r="G28" s="44"/>
-      <c r="H28" s="93"/>
-      <c r="I28" s="46"/>
-      <c r="J28" s="44"/>
-      <c r="K28" s="93"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="44"/>
-      <c r="N28" s="93"/>
-      <c r="O28" s="46"/>
-      <c r="P28" s="44"/>
-      <c r="Q28" s="45"/>
-      <c r="R28" s="45"/>
-      <c r="S28" s="46"/>
+      <c r="C28" s="73"/>
+      <c r="D28" s="74"/>
+      <c r="E28" s="74"/>
+      <c r="F28" s="75"/>
+      <c r="G28" s="73"/>
+      <c r="H28" s="74"/>
+      <c r="I28" s="75"/>
+      <c r="J28" s="73"/>
+      <c r="K28" s="74"/>
+      <c r="L28" s="75"/>
+      <c r="M28" s="73"/>
+      <c r="N28" s="74"/>
+      <c r="O28" s="75"/>
+      <c r="P28" s="95"/>
+      <c r="Q28" s="95"/>
+      <c r="R28" s="95"/>
+      <c r="S28" s="75"/>
       <c r="T28" s="6"/>
     </row>
     <row r="29" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B29" s="4"/>
-      <c r="C29" s="47"/>
-      <c r="D29" s="48"/>
-      <c r="E29" s="48"/>
-      <c r="F29" s="49"/>
-      <c r="G29" s="47"/>
-      <c r="H29" s="48"/>
-      <c r="I29" s="49"/>
-      <c r="J29" s="47"/>
-      <c r="K29" s="48"/>
-      <c r="L29" s="49"/>
-      <c r="M29" s="47"/>
-      <c r="N29" s="48"/>
-      <c r="O29" s="49"/>
-      <c r="P29" s="47"/>
-      <c r="Q29" s="48"/>
-      <c r="R29" s="48"/>
-      <c r="S29" s="49"/>
+      <c r="C29" s="76"/>
+      <c r="D29" s="77"/>
+      <c r="E29" s="77"/>
+      <c r="F29" s="78"/>
+      <c r="G29" s="76"/>
+      <c r="H29" s="77"/>
+      <c r="I29" s="78"/>
+      <c r="J29" s="76"/>
+      <c r="K29" s="77"/>
+      <c r="L29" s="78"/>
+      <c r="M29" s="76"/>
+      <c r="N29" s="77"/>
+      <c r="O29" s="78"/>
+      <c r="P29" s="77"/>
+      <c r="Q29" s="77"/>
+      <c r="R29" s="77"/>
+      <c r="S29" s="78"/>
       <c r="T29" s="6"/>
     </row>
     <row r="30" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B30" s="4"/>
-      <c r="C30" s="41" t="s">
+      <c r="C30" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D30" s="42"/>
-      <c r="E30" s="42"/>
-      <c r="F30" s="43"/>
-      <c r="G30" s="41" t="s">
+      <c r="D30" s="71"/>
+      <c r="E30" s="71"/>
+      <c r="F30" s="72"/>
+      <c r="G30" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H30" s="42"/>
-      <c r="I30" s="43"/>
-      <c r="J30" s="41" t="s">
+      <c r="H30" s="71"/>
+      <c r="I30" s="72"/>
+      <c r="J30" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K30" s="42"/>
-      <c r="L30" s="43"/>
-      <c r="M30" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N30" s="42"/>
-      <c r="O30" s="43"/>
-      <c r="P30" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q30" s="42"/>
-      <c r="R30" s="42"/>
-      <c r="S30" s="43"/>
+      <c r="K30" s="71"/>
+      <c r="L30" s="72"/>
+      <c r="M30" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N30" s="71"/>
+      <c r="O30" s="72"/>
+      <c r="P30" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q30" s="71"/>
+      <c r="R30" s="71"/>
+      <c r="S30" s="72"/>
       <c r="T30" s="6"/>
     </row>
     <row r="31" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B31" s="4"/>
-      <c r="C31" s="44"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="46"/>
-      <c r="G31" s="44"/>
-      <c r="H31" s="93"/>
-      <c r="I31" s="46"/>
-      <c r="J31" s="44"/>
-      <c r="K31" s="93"/>
-      <c r="L31" s="46"/>
-      <c r="M31" s="44"/>
-      <c r="N31" s="93"/>
-      <c r="O31" s="46"/>
-      <c r="P31" s="44"/>
-      <c r="Q31" s="45"/>
-      <c r="R31" s="45"/>
-      <c r="S31" s="46"/>
+      <c r="C31" s="73"/>
+      <c r="D31" s="74"/>
+      <c r="E31" s="74"/>
+      <c r="F31" s="75"/>
+      <c r="G31" s="73"/>
+      <c r="H31" s="74"/>
+      <c r="I31" s="75"/>
+      <c r="J31" s="73"/>
+      <c r="K31" s="74"/>
+      <c r="L31" s="75"/>
+      <c r="M31" s="73"/>
+      <c r="N31" s="74"/>
+      <c r="O31" s="75"/>
+      <c r="P31" s="95"/>
+      <c r="Q31" s="95"/>
+      <c r="R31" s="95"/>
+      <c r="S31" s="75"/>
       <c r="T31" s="6"/>
     </row>
     <row r="32" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B32" s="4"/>
-      <c r="C32" s="47"/>
-      <c r="D32" s="48"/>
-      <c r="E32" s="48"/>
-      <c r="F32" s="49"/>
-      <c r="G32" s="47"/>
-      <c r="H32" s="48"/>
-      <c r="I32" s="49"/>
-      <c r="J32" s="47"/>
-      <c r="K32" s="48"/>
-      <c r="L32" s="49"/>
-      <c r="M32" s="47"/>
-      <c r="N32" s="48"/>
-      <c r="O32" s="49"/>
-      <c r="P32" s="47"/>
-      <c r="Q32" s="48"/>
-      <c r="R32" s="48"/>
-      <c r="S32" s="49"/>
+      <c r="C32" s="76"/>
+      <c r="D32" s="77"/>
+      <c r="E32" s="77"/>
+      <c r="F32" s="78"/>
+      <c r="G32" s="76"/>
+      <c r="H32" s="77"/>
+      <c r="I32" s="78"/>
+      <c r="J32" s="76"/>
+      <c r="K32" s="77"/>
+      <c r="L32" s="78"/>
+      <c r="M32" s="76"/>
+      <c r="N32" s="77"/>
+      <c r="O32" s="78"/>
+      <c r="P32" s="77"/>
+      <c r="Q32" s="77"/>
+      <c r="R32" s="77"/>
+      <c r="S32" s="78"/>
       <c r="T32" s="6"/>
     </row>
     <row r="33" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B33" s="4"/>
-      <c r="C33" s="41" t="s">
+      <c r="C33" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D33" s="42"/>
-      <c r="E33" s="42"/>
-      <c r="F33" s="43"/>
-      <c r="G33" s="41" t="s">
+      <c r="D33" s="71"/>
+      <c r="E33" s="71"/>
+      <c r="F33" s="72"/>
+      <c r="G33" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H33" s="42"/>
-      <c r="I33" s="43"/>
-      <c r="J33" s="41" t="s">
+      <c r="H33" s="71"/>
+      <c r="I33" s="72"/>
+      <c r="J33" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K33" s="42"/>
-      <c r="L33" s="43"/>
-      <c r="M33" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N33" s="42"/>
-      <c r="O33" s="43"/>
-      <c r="P33" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q33" s="42"/>
-      <c r="R33" s="42"/>
-      <c r="S33" s="43"/>
+      <c r="K33" s="71"/>
+      <c r="L33" s="72"/>
+      <c r="M33" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N33" s="71"/>
+      <c r="O33" s="72"/>
+      <c r="P33" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q33" s="71"/>
+      <c r="R33" s="71"/>
+      <c r="S33" s="72"/>
       <c r="T33" s="6"/>
     </row>
     <row r="34" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B34" s="4"/>
-      <c r="C34" s="44"/>
-      <c r="D34" s="45"/>
-      <c r="E34" s="45"/>
-      <c r="F34" s="46"/>
-      <c r="G34" s="44"/>
-      <c r="H34" s="93"/>
-      <c r="I34" s="46"/>
-      <c r="J34" s="44"/>
-      <c r="K34" s="93"/>
-      <c r="L34" s="46"/>
-      <c r="M34" s="44"/>
-      <c r="N34" s="93"/>
-      <c r="O34" s="46"/>
-      <c r="P34" s="44"/>
-      <c r="Q34" s="45"/>
-      <c r="R34" s="45"/>
-      <c r="S34" s="46"/>
+      <c r="C34" s="73"/>
+      <c r="D34" s="74"/>
+      <c r="E34" s="74"/>
+      <c r="F34" s="75"/>
+      <c r="G34" s="73"/>
+      <c r="H34" s="74"/>
+      <c r="I34" s="75"/>
+      <c r="J34" s="73"/>
+      <c r="K34" s="74"/>
+      <c r="L34" s="75"/>
+      <c r="M34" s="73"/>
+      <c r="N34" s="74"/>
+      <c r="O34" s="75"/>
+      <c r="P34" s="95"/>
+      <c r="Q34" s="95"/>
+      <c r="R34" s="95"/>
+      <c r="S34" s="75"/>
       <c r="T34" s="6"/>
     </row>
     <row r="35" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B35" s="4"/>
-      <c r="C35" s="47"/>
-      <c r="D35" s="48"/>
-      <c r="E35" s="48"/>
-      <c r="F35" s="49"/>
-      <c r="G35" s="47"/>
-      <c r="H35" s="48"/>
-      <c r="I35" s="49"/>
-      <c r="J35" s="47"/>
-      <c r="K35" s="48"/>
-      <c r="L35" s="49"/>
-      <c r="M35" s="47"/>
-      <c r="N35" s="48"/>
-      <c r="O35" s="49"/>
-      <c r="P35" s="47"/>
-      <c r="Q35" s="48"/>
-      <c r="R35" s="48"/>
-      <c r="S35" s="49"/>
+      <c r="C35" s="76"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="77"/>
+      <c r="F35" s="78"/>
+      <c r="G35" s="76"/>
+      <c r="H35" s="77"/>
+      <c r="I35" s="78"/>
+      <c r="J35" s="76"/>
+      <c r="K35" s="77"/>
+      <c r="L35" s="78"/>
+      <c r="M35" s="76"/>
+      <c r="N35" s="77"/>
+      <c r="O35" s="78"/>
+      <c r="P35" s="77"/>
+      <c r="Q35" s="77"/>
+      <c r="R35" s="77"/>
+      <c r="S35" s="78"/>
       <c r="T35" s="6"/>
     </row>
     <row r="36" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="4"/>
-      <c r="C36" s="41" t="s">
+      <c r="C36" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D36" s="42"/>
-      <c r="E36" s="42"/>
-      <c r="F36" s="43"/>
-      <c r="G36" s="41" t="s">
+      <c r="D36" s="71"/>
+      <c r="E36" s="71"/>
+      <c r="F36" s="72"/>
+      <c r="G36" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H36" s="42"/>
-      <c r="I36" s="43"/>
-      <c r="J36" s="41" t="s">
+      <c r="H36" s="71"/>
+      <c r="I36" s="72"/>
+      <c r="J36" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K36" s="42"/>
-      <c r="L36" s="43"/>
-      <c r="M36" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N36" s="42"/>
-      <c r="O36" s="43"/>
-      <c r="P36" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q36" s="42"/>
-      <c r="R36" s="42"/>
-      <c r="S36" s="43"/>
+      <c r="K36" s="71"/>
+      <c r="L36" s="72"/>
+      <c r="M36" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N36" s="71"/>
+      <c r="O36" s="72"/>
+      <c r="P36" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q36" s="71"/>
+      <c r="R36" s="71"/>
+      <c r="S36" s="72"/>
       <c r="T36" s="6"/>
     </row>
     <row r="37" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B37" s="4"/>
-      <c r="C37" s="44"/>
-      <c r="D37" s="45"/>
-      <c r="E37" s="45"/>
-      <c r="F37" s="46"/>
-      <c r="G37" s="44"/>
-      <c r="H37" s="93"/>
-      <c r="I37" s="46"/>
-      <c r="J37" s="44"/>
-      <c r="K37" s="93"/>
-      <c r="L37" s="46"/>
-      <c r="M37" s="44"/>
-      <c r="N37" s="93"/>
-      <c r="O37" s="46"/>
-      <c r="P37" s="44"/>
-      <c r="Q37" s="45"/>
-      <c r="R37" s="45"/>
-      <c r="S37" s="46"/>
+      <c r="C37" s="73"/>
+      <c r="D37" s="74"/>
+      <c r="E37" s="74"/>
+      <c r="F37" s="75"/>
+      <c r="G37" s="73"/>
+      <c r="H37" s="74"/>
+      <c r="I37" s="75"/>
+      <c r="J37" s="73"/>
+      <c r="K37" s="74"/>
+      <c r="L37" s="75"/>
+      <c r="M37" s="73"/>
+      <c r="N37" s="74"/>
+      <c r="O37" s="75"/>
+      <c r="P37" s="95"/>
+      <c r="Q37" s="95"/>
+      <c r="R37" s="95"/>
+      <c r="S37" s="75"/>
       <c r="T37" s="6"/>
     </row>
     <row r="38" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B38" s="4"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="48"/>
-      <c r="E38" s="48"/>
-      <c r="F38" s="49"/>
-      <c r="G38" s="47"/>
-      <c r="H38" s="48"/>
-      <c r="I38" s="49"/>
-      <c r="J38" s="47"/>
-      <c r="K38" s="48"/>
-      <c r="L38" s="49"/>
-      <c r="M38" s="47"/>
-      <c r="N38" s="48"/>
-      <c r="O38" s="49"/>
-      <c r="P38" s="47"/>
-      <c r="Q38" s="48"/>
-      <c r="R38" s="48"/>
-      <c r="S38" s="49"/>
+      <c r="C38" s="76"/>
+      <c r="D38" s="77"/>
+      <c r="E38" s="77"/>
+      <c r="F38" s="78"/>
+      <c r="G38" s="76"/>
+      <c r="H38" s="77"/>
+      <c r="I38" s="78"/>
+      <c r="J38" s="76"/>
+      <c r="K38" s="77"/>
+      <c r="L38" s="78"/>
+      <c r="M38" s="76"/>
+      <c r="N38" s="77"/>
+      <c r="O38" s="78"/>
+      <c r="P38" s="77"/>
+      <c r="Q38" s="77"/>
+      <c r="R38" s="77"/>
+      <c r="S38" s="78"/>
       <c r="T38" s="6"/>
     </row>
     <row r="39" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B39" s="4"/>
-      <c r="C39" s="41" t="s">
+      <c r="C39" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="D39" s="42"/>
-      <c r="E39" s="42"/>
-      <c r="F39" s="43"/>
-      <c r="G39" s="41" t="s">
+      <c r="D39" s="71"/>
+      <c r="E39" s="71"/>
+      <c r="F39" s="72"/>
+      <c r="G39" s="70" t="s">
         <v>3</v>
       </c>
-      <c r="H39" s="42"/>
-      <c r="I39" s="43"/>
-      <c r="J39" s="41" t="s">
+      <c r="H39" s="71"/>
+      <c r="I39" s="72"/>
+      <c r="J39" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="K39" s="42"/>
-      <c r="L39" s="43"/>
-      <c r="M39" s="41" t="s">
-        <v>36</v>
-      </c>
-      <c r="N39" s="42"/>
-      <c r="O39" s="43"/>
-      <c r="P39" s="41" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q39" s="42"/>
-      <c r="R39" s="42"/>
-      <c r="S39" s="43"/>
+      <c r="K39" s="71"/>
+      <c r="L39" s="72"/>
+      <c r="M39" s="70" t="s">
+        <v>32</v>
+      </c>
+      <c r="N39" s="71"/>
+      <c r="O39" s="72"/>
+      <c r="P39" s="71" t="s">
+        <v>45</v>
+      </c>
+      <c r="Q39" s="71"/>
+      <c r="R39" s="71"/>
+      <c r="S39" s="72"/>
       <c r="T39" s="6"/>
     </row>
     <row r="40" spans="2:20" ht="13.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B40" s="4"/>
-      <c r="C40" s="44"/>
-      <c r="D40" s="45"/>
-      <c r="E40" s="45"/>
-      <c r="F40" s="46"/>
-      <c r="G40" s="44"/>
-      <c r="H40" s="93"/>
-      <c r="I40" s="46"/>
-      <c r="J40" s="44"/>
-      <c r="K40" s="93"/>
-      <c r="L40" s="46"/>
-      <c r="M40" s="44"/>
-      <c r="N40" s="93"/>
-      <c r="O40" s="46"/>
-      <c r="P40" s="44"/>
-      <c r="Q40" s="45"/>
-      <c r="R40" s="45"/>
-      <c r="S40" s="46"/>
+      <c r="C40" s="73"/>
+      <c r="D40" s="74"/>
+      <c r="E40" s="74"/>
+      <c r="F40" s="75"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="74"/>
+      <c r="I40" s="75"/>
+      <c r="J40" s="73"/>
+      <c r="K40" s="74"/>
+      <c r="L40" s="75"/>
+      <c r="M40" s="73"/>
+      <c r="N40" s="74"/>
+      <c r="O40" s="75"/>
+      <c r="P40" s="95"/>
+      <c r="Q40" s="95"/>
+      <c r="R40" s="95"/>
+      <c r="S40" s="75"/>
       <c r="T40" s="6"/>
     </row>
     <row r="41" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B41" s="4"/>
-      <c r="C41" s="47"/>
-      <c r="D41" s="48"/>
-      <c r="E41" s="48"/>
-      <c r="F41" s="49"/>
-      <c r="G41" s="47"/>
-      <c r="H41" s="48"/>
-      <c r="I41" s="49"/>
-      <c r="J41" s="47"/>
-      <c r="K41" s="48"/>
-      <c r="L41" s="49"/>
-      <c r="M41" s="47"/>
-      <c r="N41" s="48"/>
-      <c r="O41" s="49"/>
-      <c r="P41" s="47"/>
-      <c r="Q41" s="48"/>
-      <c r="R41" s="48"/>
-      <c r="S41" s="49"/>
+      <c r="C41" s="76"/>
+      <c r="D41" s="77"/>
+      <c r="E41" s="77"/>
+      <c r="F41" s="78"/>
+      <c r="G41" s="76"/>
+      <c r="H41" s="77"/>
+      <c r="I41" s="78"/>
+      <c r="J41" s="76"/>
+      <c r="K41" s="77"/>
+      <c r="L41" s="78"/>
+      <c r="M41" s="76"/>
+      <c r="N41" s="77"/>
+      <c r="O41" s="78"/>
+      <c r="P41" s="77"/>
+      <c r="Q41" s="77"/>
+      <c r="R41" s="77"/>
+      <c r="S41" s="78"/>
       <c r="T41" s="6"/>
     </row>
     <row r="42" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B42" s="4"/>
       <c r="C42" s="5"/>
-      <c r="D42" s="5"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
-      <c r="H42" s="8"/>
-      <c r="I42" s="8"/>
+      <c r="D42" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E42" s="56"/>
+      <c r="F42" s="56"/>
+      <c r="G42" s="56"/>
+      <c r="H42" s="56"/>
+      <c r="I42" s="56"/>
       <c r="J42" s="8"/>
       <c r="K42" s="8"/>
       <c r="L42" s="8"/>
-      <c r="M42" s="71" t="s">
-        <v>32</v>
-      </c>
-      <c r="N42" s="72"/>
-      <c r="O42" s="73"/>
-      <c r="P42" s="50" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q42" s="51"/>
-      <c r="R42" s="51"/>
-      <c r="S42" s="52"/>
+      <c r="M42" s="50" t="s">
+        <v>31</v>
+      </c>
+      <c r="N42" s="51"/>
+      <c r="O42" s="52"/>
+      <c r="P42" s="53" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q42" s="54"/>
+      <c r="R42" s="54"/>
+      <c r="S42" s="55"/>
       <c r="T42" s="6"/>
     </row>
     <row r="43" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B43" s="4"/>
       <c r="C43" s="5"/>
-      <c r="D43" s="5"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
-      <c r="H43" s="8"/>
-      <c r="I43" s="8"/>
+      <c r="D43" s="56"/>
+      <c r="E43" s="56"/>
+      <c r="F43" s="56"/>
+      <c r="G43" s="56"/>
+      <c r="H43" s="56"/>
+      <c r="I43" s="56"/>
       <c r="J43" s="8"/>
       <c r="K43" s="8"/>
       <c r="L43" s="8"/>
-      <c r="M43" s="90" t="s">
-        <v>35</v>
-      </c>
-      <c r="N43" s="91"/>
-      <c r="O43" s="92"/>
-      <c r="P43" s="87" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q43" s="88"/>
-      <c r="R43" s="88"/>
-      <c r="S43" s="89"/>
+      <c r="M43" s="43" t="s">
+        <v>34</v>
+      </c>
+      <c r="N43" s="44"/>
+      <c r="O43" s="45"/>
+      <c r="P43" s="46" t="s">
+        <v>36</v>
+      </c>
+      <c r="Q43" s="47"/>
+      <c r="R43" s="47"/>
+      <c r="S43" s="48"/>
       <c r="T43" s="6"/>
     </row>
     <row r="44" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B44" s="4"/>
       <c r="C44" s="8"/>
-      <c r="D44" s="70" t="s">
-        <v>31</v>
-      </c>
-      <c r="E44" s="70"/>
-      <c r="F44" s="70"/>
-      <c r="G44" s="70"/>
-      <c r="H44" s="70"/>
-      <c r="I44" s="70"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
       <c r="J44" s="39"/>
       <c r="K44" s="5"/>
       <c r="L44" s="5"/>
-      <c r="M44" s="90" t="s">
+      <c r="M44" s="43" t="s">
         <v>11</v>
       </c>
-      <c r="N44" s="91"/>
-      <c r="O44" s="92"/>
-      <c r="P44" s="87" t="s">
+      <c r="N44" s="44"/>
+      <c r="O44" s="45"/>
+      <c r="P44" s="46" t="s">
         <v>5</v>
       </c>
-      <c r="Q44" s="88"/>
-      <c r="R44" s="88"/>
-      <c r="S44" s="89"/>
+      <c r="Q44" s="47"/>
+      <c r="R44" s="47"/>
+      <c r="S44" s="48"/>
       <c r="T44" s="6"/>
     </row>
     <row r="45" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B45" s="4"/>
       <c r="C45" s="8"/>
-      <c r="D45" s="70"/>
-      <c r="E45" s="70"/>
-      <c r="F45" s="70"/>
-      <c r="G45" s="70"/>
-      <c r="H45" s="70"/>
-      <c r="I45" s="70"/>
+      <c r="D45" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E45" s="56"/>
+      <c r="F45" s="56"/>
+      <c r="G45" s="56"/>
+      <c r="H45" s="56"/>
+      <c r="I45" s="56"/>
       <c r="J45" s="39"/>
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
-      <c r="M45" s="90" t="s">
+      <c r="M45" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="N45" s="91"/>
-      <c r="O45" s="92"/>
-      <c r="P45" s="87" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q45" s="88"/>
-      <c r="R45" s="88"/>
-      <c r="S45" s="89"/>
+      <c r="N45" s="44"/>
+      <c r="O45" s="45"/>
+      <c r="P45" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q45" s="47"/>
+      <c r="R45" s="47"/>
+      <c r="S45" s="48"/>
       <c r="T45" s="6"/>
     </row>
     <row r="46" spans="2:20" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B46" s="4"/>
       <c r="C46" s="38"/>
-      <c r="D46" s="38"/>
-      <c r="E46" s="38"/>
-      <c r="F46" s="38"/>
-      <c r="G46" s="38"/>
-      <c r="H46" s="38"/>
-      <c r="I46" s="38"/>
+      <c r="D46" s="56"/>
+      <c r="E46" s="56"/>
+      <c r="F46" s="56"/>
+      <c r="G46" s="56"/>
+      <c r="H46" s="56"/>
+      <c r="I46" s="56"/>
       <c r="J46" s="5"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
-      <c r="M46" s="90" t="s">
-        <v>41</v>
-      </c>
-      <c r="N46" s="91"/>
-      <c r="O46" s="92"/>
-      <c r="P46" s="87" t="s">
-        <v>42</v>
-      </c>
-      <c r="Q46" s="88"/>
-      <c r="R46" s="88"/>
-      <c r="S46" s="89"/>
+      <c r="M46" s="43" t="s">
+        <v>39</v>
+      </c>
+      <c r="N46" s="44"/>
+      <c r="O46" s="45"/>
+      <c r="P46" s="46" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q46" s="47"/>
+      <c r="R46" s="47"/>
+      <c r="S46" s="48"/>
       <c r="T46" s="6"/>
     </row>
     <row r="47" spans="2:20" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B47" s="4"/>
       <c r="C47" s="8"/>
-      <c r="D47" s="70" t="s">
-        <v>31</v>
-      </c>
-      <c r="E47" s="70"/>
-      <c r="F47" s="70"/>
-      <c r="G47" s="70"/>
-      <c r="H47" s="70"/>
-      <c r="I47" s="70"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="38"/>
+      <c r="G47" s="38"/>
+      <c r="H47" s="38"/>
+      <c r="I47" s="38"/>
       <c r="J47" s="39"/>
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
@@ -2446,100 +2459,102 @@
     <row r="48" spans="2:20" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B48" s="4"/>
       <c r="C48" s="8"/>
-      <c r="D48" s="70"/>
-      <c r="E48" s="70"/>
-      <c r="F48" s="70"/>
-      <c r="G48" s="70"/>
-      <c r="H48" s="70"/>
-      <c r="I48" s="70"/>
+      <c r="D48" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E48" s="56"/>
+      <c r="F48" s="56"/>
+      <c r="G48" s="56"/>
+      <c r="H48" s="56"/>
+      <c r="I48" s="56"/>
       <c r="J48" s="39"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
-      <c r="M48" s="94"/>
-      <c r="N48" s="94"/>
-      <c r="O48" s="94"/>
-      <c r="P48" s="94"/>
-      <c r="Q48" s="94"/>
-      <c r="R48" s="94"/>
-      <c r="S48" s="94"/>
+      <c r="M48" s="41"/>
+      <c r="N48" s="41"/>
+      <c r="O48" s="41"/>
+      <c r="P48" s="41"/>
+      <c r="Q48" s="41"/>
+      <c r="R48" s="41"/>
+      <c r="S48" s="41"/>
       <c r="T48" s="6"/>
     </row>
     <row r="49" spans="2:20" ht="7.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B49" s="4"/>
       <c r="C49" s="38"/>
-      <c r="D49" s="38"/>
-      <c r="E49" s="38"/>
-      <c r="F49" s="38"/>
-      <c r="G49" s="38"/>
-      <c r="H49" s="38"/>
-      <c r="I49" s="38"/>
+      <c r="D49" s="56"/>
+      <c r="E49" s="56"/>
+      <c r="F49" s="56"/>
+      <c r="G49" s="56"/>
+      <c r="H49" s="56"/>
+      <c r="I49" s="56"/>
       <c r="J49" s="5"/>
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
-      <c r="M49" s="94"/>
-      <c r="N49" s="94"/>
-      <c r="O49" s="94"/>
-      <c r="P49" s="94"/>
-      <c r="Q49" s="94"/>
-      <c r="R49" s="94"/>
-      <c r="S49" s="94"/>
+      <c r="M49" s="41"/>
+      <c r="N49" s="41"/>
+      <c r="O49" s="41"/>
+      <c r="P49" s="41"/>
+      <c r="Q49" s="41"/>
+      <c r="R49" s="41"/>
+      <c r="S49" s="41"/>
       <c r="T49" s="6"/>
     </row>
     <row r="50" spans="2:20" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B50" s="4"/>
       <c r="C50" s="8"/>
-      <c r="D50" s="70" t="s">
-        <v>31</v>
-      </c>
-      <c r="E50" s="70"/>
-      <c r="F50" s="70"/>
-      <c r="G50" s="70"/>
-      <c r="H50" s="70"/>
-      <c r="I50" s="70"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38"/>
+      <c r="F50" s="38"/>
+      <c r="G50" s="38"/>
+      <c r="H50" s="38"/>
+      <c r="I50" s="38"/>
       <c r="J50" s="39"/>
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
-      <c r="M50" s="95"/>
-      <c r="N50" s="95"/>
-      <c r="O50" s="95"/>
-      <c r="P50" s="95"/>
-      <c r="Q50" s="95"/>
-      <c r="R50" s="95"/>
-      <c r="S50" s="95"/>
+      <c r="M50" s="42"/>
+      <c r="N50" s="42"/>
+      <c r="O50" s="42"/>
+      <c r="P50" s="42"/>
+      <c r="Q50" s="42"/>
+      <c r="R50" s="42"/>
+      <c r="S50" s="42"/>
       <c r="T50" s="6"/>
     </row>
     <row r="51" spans="2:20" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B51" s="4"/>
       <c r="C51" s="8"/>
-      <c r="D51" s="70"/>
-      <c r="E51" s="70"/>
-      <c r="F51" s="70"/>
-      <c r="G51" s="70"/>
-      <c r="H51" s="70"/>
-      <c r="I51" s="70"/>
+      <c r="D51" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E51" s="56"/>
+      <c r="F51" s="56"/>
+      <c r="G51" s="56"/>
+      <c r="H51" s="56"/>
+      <c r="I51" s="56"/>
       <c r="J51" s="39"/>
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
-      <c r="M51" s="77" t="s">
+      <c r="M51" s="60" t="s">
         <v>1</v>
       </c>
-      <c r="N51" s="77"/>
-      <c r="O51" s="77"/>
-      <c r="P51" s="77"/>
-      <c r="Q51" s="77"/>
-      <c r="R51" s="77"/>
-      <c r="S51" s="77"/>
+      <c r="N51" s="60"/>
+      <c r="O51" s="60"/>
+      <c r="P51" s="60"/>
+      <c r="Q51" s="60"/>
+      <c r="R51" s="60"/>
+      <c r="S51" s="60"/>
       <c r="T51" s="6"/>
     </row>
     <row r="52" spans="2:20" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B52" s="4"/>
       <c r="C52" s="38"/>
-      <c r="D52" s="38"/>
-      <c r="E52" s="38"/>
-      <c r="F52" s="38"/>
-      <c r="G52" s="38"/>
-      <c r="H52" s="38"/>
-      <c r="I52" s="38"/>
+      <c r="D52" s="56"/>
+      <c r="E52" s="56"/>
+      <c r="F52" s="56"/>
+      <c r="G52" s="56"/>
+      <c r="H52" s="56"/>
+      <c r="I52" s="56"/>
       <c r="J52" s="5"/>
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
@@ -2555,70 +2570,70 @@
     <row r="53" spans="2:20" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B53" s="4"/>
       <c r="C53" s="8"/>
-      <c r="D53" s="70" t="s">
-        <v>31</v>
-      </c>
-      <c r="E53" s="70"/>
-      <c r="F53" s="70"/>
-      <c r="G53" s="70"/>
-      <c r="H53" s="70"/>
-      <c r="I53" s="70"/>
+      <c r="D53" s="39"/>
+      <c r="E53" s="39"/>
+      <c r="F53" s="39"/>
+      <c r="G53" s="39"/>
+      <c r="H53" s="39"/>
+      <c r="I53" s="39"/>
       <c r="J53" s="39"/>
       <c r="K53" s="5"/>
       <c r="L53" s="5"/>
-      <c r="M53" s="78" t="s">
-        <v>29</v>
-      </c>
-      <c r="N53" s="79"/>
-      <c r="O53" s="80"/>
-      <c r="P53" s="78" t="s">
+      <c r="M53" s="61" t="s">
+        <v>28</v>
+      </c>
+      <c r="N53" s="62"/>
+      <c r="O53" s="63"/>
+      <c r="P53" s="61" t="s">
         <v>6</v>
       </c>
-      <c r="Q53" s="79"/>
-      <c r="R53" s="79"/>
-      <c r="S53" s="80"/>
+      <c r="Q53" s="62"/>
+      <c r="R53" s="62"/>
+      <c r="S53" s="63"/>
       <c r="T53" s="6"/>
     </row>
-    <row r="54" spans="2:20" x14ac:dyDescent="0.25">
+    <row r="54" spans="2:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B54" s="4"/>
       <c r="C54" s="8"/>
-      <c r="D54" s="70"/>
-      <c r="E54" s="70"/>
-      <c r="F54" s="70"/>
-      <c r="G54" s="70"/>
-      <c r="H54" s="70"/>
-      <c r="I54" s="70"/>
+      <c r="D54" s="56" t="s">
+        <v>30</v>
+      </c>
+      <c r="E54" s="56"/>
+      <c r="F54" s="56"/>
+      <c r="G54" s="56"/>
+      <c r="H54" s="56"/>
+      <c r="I54" s="56"/>
       <c r="J54" s="39"/>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
-      <c r="M54" s="81"/>
-      <c r="N54" s="82"/>
-      <c r="O54" s="83"/>
-      <c r="P54" s="81"/>
-      <c r="Q54" s="82"/>
-      <c r="R54" s="82"/>
-      <c r="S54" s="83"/>
+      <c r="M54" s="64"/>
+      <c r="N54" s="65"/>
+      <c r="O54" s="66"/>
+      <c r="P54" s="64"/>
+      <c r="Q54" s="65"/>
+      <c r="R54" s="65"/>
+      <c r="S54" s="66"/>
       <c r="T54" s="6"/>
     </row>
     <row r="55" spans="2:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B55" s="4"/>
       <c r="C55" s="5"/>
-      <c r="D55" s="5"/>
-      <c r="E55" s="5"/>
-      <c r="F55" s="5"/>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
+      <c r="D55" s="56"/>
+      <c r="E55" s="56"/>
+      <c r="F55" s="56"/>
+      <c r="G55" s="56"/>
+      <c r="H55" s="56"/>
+      <c r="I55" s="56"/>
       <c r="J55" s="5"/>
       <c r="K55" s="5"/>
       <c r="L55" s="5"/>
-      <c r="M55" s="84"/>
-      <c r="N55" s="85"/>
-      <c r="O55" s="86"/>
-      <c r="P55" s="84"/>
-      <c r="Q55" s="85"/>
-      <c r="R55" s="85"/>
-      <c r="S55" s="86"/>
+      <c r="M55" s="67"/>
+      <c r="N55" s="68"/>
+      <c r="O55" s="69"/>
+      <c r="P55" s="67"/>
+      <c r="Q55" s="68"/>
+      <c r="R55" s="68"/>
+      <c r="S55" s="69"/>
       <c r="T55" s="6"/>
     </row>
     <row r="56" spans="2:20" ht="8.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2644,6 +2659,61 @@
     </row>
   </sheetData>
   <mergeCells count="70">
+    <mergeCell ref="P39:S41"/>
+    <mergeCell ref="P22:S23"/>
+    <mergeCell ref="P27:S29"/>
+    <mergeCell ref="P30:S32"/>
+    <mergeCell ref="M33:O35"/>
+    <mergeCell ref="P33:S35"/>
+    <mergeCell ref="M36:O38"/>
+    <mergeCell ref="P36:S38"/>
+    <mergeCell ref="G24:I26"/>
+    <mergeCell ref="G30:I32"/>
+    <mergeCell ref="D54:I55"/>
+    <mergeCell ref="M22:O23"/>
+    <mergeCell ref="M24:O26"/>
+    <mergeCell ref="M27:O29"/>
+    <mergeCell ref="M30:O32"/>
+    <mergeCell ref="M39:O41"/>
+    <mergeCell ref="C36:F38"/>
+    <mergeCell ref="C39:F41"/>
+    <mergeCell ref="C27:F29"/>
+    <mergeCell ref="G36:I38"/>
+    <mergeCell ref="G39:I41"/>
+    <mergeCell ref="G27:I29"/>
+    <mergeCell ref="C33:F35"/>
+    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J36:L38"/>
+    <mergeCell ref="J27:L29"/>
+    <mergeCell ref="J24:L26"/>
+    <mergeCell ref="J30:L32"/>
+    <mergeCell ref="J33:L35"/>
+    <mergeCell ref="D6:H8"/>
+    <mergeCell ref="G16:I17"/>
+    <mergeCell ref="G9:H9"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="O8:R9"/>
+    <mergeCell ref="L14:N14"/>
+    <mergeCell ref="O14:Q14"/>
+    <mergeCell ref="O15:Q15"/>
+    <mergeCell ref="O16:Q16"/>
+    <mergeCell ref="O17:Q17"/>
+    <mergeCell ref="E10:G10"/>
+    <mergeCell ref="J6:N7"/>
+    <mergeCell ref="J8:N9"/>
+    <mergeCell ref="D42:I43"/>
+    <mergeCell ref="D45:I46"/>
+    <mergeCell ref="D48:I49"/>
+    <mergeCell ref="D51:I52"/>
+    <mergeCell ref="G22:I23"/>
+    <mergeCell ref="C22:F23"/>
+    <mergeCell ref="J22:L23"/>
+    <mergeCell ref="M51:S51"/>
+    <mergeCell ref="M53:O55"/>
+    <mergeCell ref="P53:S55"/>
+    <mergeCell ref="C24:F26"/>
+    <mergeCell ref="C30:F32"/>
+    <mergeCell ref="G33:I35"/>
     <mergeCell ref="M46:O46"/>
     <mergeCell ref="P46:S46"/>
     <mergeCell ref="L15:N15"/>
@@ -2657,71 +2727,17 @@
     <mergeCell ref="P42:S42"/>
     <mergeCell ref="M43:O43"/>
     <mergeCell ref="P43:S43"/>
-    <mergeCell ref="D44:I45"/>
-    <mergeCell ref="D47:I48"/>
-    <mergeCell ref="D50:I51"/>
-    <mergeCell ref="D53:I54"/>
-    <mergeCell ref="P22:S23"/>
-    <mergeCell ref="G22:I23"/>
-    <mergeCell ref="C22:F23"/>
-    <mergeCell ref="M22:O23"/>
-    <mergeCell ref="J22:L23"/>
-    <mergeCell ref="M51:S51"/>
-    <mergeCell ref="M53:O55"/>
-    <mergeCell ref="P53:S55"/>
-    <mergeCell ref="C24:F26"/>
-    <mergeCell ref="C30:F32"/>
-    <mergeCell ref="D6:H8"/>
-    <mergeCell ref="G16:I17"/>
-    <mergeCell ref="G9:H9"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="O8:R9"/>
-    <mergeCell ref="L14:N14"/>
-    <mergeCell ref="O14:Q14"/>
-    <mergeCell ref="O15:Q15"/>
-    <mergeCell ref="O16:Q16"/>
-    <mergeCell ref="O17:Q17"/>
-    <mergeCell ref="E10:G10"/>
-    <mergeCell ref="G33:I35"/>
-    <mergeCell ref="G14:I15"/>
-    <mergeCell ref="J6:N7"/>
-    <mergeCell ref="J8:N9"/>
-    <mergeCell ref="G18:I18"/>
+    <mergeCell ref="J39:L41"/>
     <mergeCell ref="P24:S26"/>
-    <mergeCell ref="P30:S32"/>
-    <mergeCell ref="P33:S35"/>
-    <mergeCell ref="P36:S38"/>
-    <mergeCell ref="P39:S41"/>
-    <mergeCell ref="P27:S29"/>
-    <mergeCell ref="J36:L38"/>
-    <mergeCell ref="J39:L41"/>
-    <mergeCell ref="M36:O38"/>
-    <mergeCell ref="M39:O41"/>
-    <mergeCell ref="J27:L29"/>
-    <mergeCell ref="M24:O26"/>
-    <mergeCell ref="M30:O32"/>
-    <mergeCell ref="M33:O35"/>
-    <mergeCell ref="C36:F38"/>
-    <mergeCell ref="C39:F41"/>
-    <mergeCell ref="C27:F29"/>
-    <mergeCell ref="G36:I38"/>
-    <mergeCell ref="G39:I41"/>
-    <mergeCell ref="G27:I29"/>
-    <mergeCell ref="M27:O29"/>
-    <mergeCell ref="C33:F35"/>
-    <mergeCell ref="J24:L26"/>
-    <mergeCell ref="J30:L32"/>
-    <mergeCell ref="J33:L35"/>
-    <mergeCell ref="G24:I26"/>
-    <mergeCell ref="G30:I32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
   <drawing r:id="rId2"/>
-  <webPublishItems count="3">
+  <webPublishItems count="4">
     <webPublishItem id="30780" divId="OrdenCompra_30780" sourceType="printArea" destinationFile="D:\Dropbox (Personal)\Proyectos\Urbano\app\templates\Recibo.htm" autoRepublish="1"/>
     <webPublishItem id="17780" divId="Recibo_17780" sourceType="printArea" destinationFile="D:\Dropbox (Personal)\Proyectos\Urbano\Docs\Recibo.htm" autoRepublish="1"/>
     <webPublishItem id="30799" divId="Recibo_30799" sourceType="printArea" destinationFile="D:\Dropbox (Personal)\Proyectos\CasaLuna\dev\templates\Recibo.htm" autoRepublish="1"/>
+    <webPublishItem id="15315" divId="Recibo_15315" sourceType="printArea" destinationFile="D:\Dropbox (Personal)\Proyectos\CasaLuna\dev\templates\Recibo.htm" autoRepublish="1"/>
   </webPublishItems>
 </worksheet>
 </file>
</xml_diff>